<commit_message>
Refactor project files and update README
</commit_message>
<xml_diff>
--- a/output/price_predictions.xlsx
+++ b/output/price_predictions.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>自動補完</t>
+          <t>入力値使用</t>
         </is>
       </c>
       <c r="U2" s="3" t="n">
@@ -775,7 +775,7 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>自動補完</t>
+          <t>入力値使用</t>
         </is>
       </c>
       <c r="U3" s="3" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>自動補完</t>
+          <t>入力値使用</t>
         </is>
       </c>
       <c r="U4" s="3" t="n">

</xml_diff>